<commit_message>
Fill the user's own Word template, generate all open reports in one run, review in Word
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/complaint-list.xlsx
+++ b/samples/complaint-list.xlsx
@@ -59,6 +59,8 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="90" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -71,12 +73,12 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>CaseId</t>
+          <t>Complaint no.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="2">
         <is>
-          <t>ReceivedDate</t>
+          <t>Date received</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="2">
@@ -86,7 +88,7 @@
       </c>
       <c r="D2" t="inlineStr" s="2">
         <is>
-          <t>ProductGroup</t>
+          <t>Product group</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="2">
@@ -106,12 +108,22 @@
       </c>
       <c r="H2" t="inlineStr" s="2">
         <is>
-          <t>SampleReceived</t>
+          <t>Sample received</t>
         </is>
       </c>
       <c r="I2" t="inlineStr" s="2">
         <is>
           <t>Description</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr" s="2">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr" s="2">
+        <is>
+          <t>Report type</t>
         </is>
       </c>
     </row>
@@ -159,6 +171,16 @@
           <t xml:space="preserve">Outer carton dented on one corner. Blister intact, no tablets missing.</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">short</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -204,6 +226,16 @@
           <t xml:space="preserve">Expiry date on the bottle label partly illegible. Carton print is readable.</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Oral Solution 100 ml</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">short</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -249,6 +281,16 @@
           <t xml:space="preserve">Two tablets in one blister show small dark specks on the surface.</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">short</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -294,6 +336,16 @@
           <t xml:space="preserve">Blister foil torn at one cavity on arrival. Capsule present and intact.</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Capsules 20 mg</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">short</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -339,6 +391,16 @@
           <t xml:space="preserve">Measuring cup missing from the carton.</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Oral Solution 100 ml</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -384,6 +446,16 @@
           <t xml:space="preserve">Carton crushed in transport. The shipping box was also damaged.</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -429,6 +501,16 @@
           <t xml:space="preserve">Customer reports a dark fibre in the cream after first opening of the tube. Sample requested.</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Cream 30 g</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -474,6 +556,16 @@
           <t xml:space="preserve">Two cartons in one shipment dented. Contents not affected.</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Capsules 20 mg</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -519,6 +611,16 @@
           <t xml:space="preserve">Patient leaflet missing from the carton.</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -562,6 +664,16 @@
       <c r="I12" t="inlineStr">
         <is>
           <t xml:space="preserve">Blister strip cracked across two cavities, one tablet broken. Customer asked for a call back on +49 30 5550 1234.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use your own Word template and Excel list, generate all open reports in one run, review in Word (#9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/complaint-list.xlsx
+++ b/samples/complaint-list.xlsx
@@ -59,6 +59,8 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="90" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -71,12 +73,12 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>CaseId</t>
+          <t>Complaint no.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="2">
         <is>
-          <t>ReceivedDate</t>
+          <t>Date received</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="2">
@@ -86,7 +88,7 @@
       </c>
       <c r="D2" t="inlineStr" s="2">
         <is>
-          <t>ProductGroup</t>
+          <t>Product group</t>
         </is>
       </c>
       <c r="E2" t="inlineStr" s="2">
@@ -106,12 +108,22 @@
       </c>
       <c r="H2" t="inlineStr" s="2">
         <is>
-          <t>SampleReceived</t>
+          <t>Sample received</t>
         </is>
       </c>
       <c r="I2" t="inlineStr" s="2">
         <is>
           <t>Description</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr" s="2">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr" s="2">
+        <is>
+          <t>Report type</t>
         </is>
       </c>
     </row>
@@ -159,6 +171,16 @@
           <t xml:space="preserve">Outer carton dented on one corner. Blister intact, no tablets missing.</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">short</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -204,6 +226,16 @@
           <t xml:space="preserve">Expiry date on the bottle label partly illegible. Carton print is readable.</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Oral Solution 100 ml</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">short</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -249,6 +281,16 @@
           <t xml:space="preserve">Two tablets in one blister show small dark specks on the surface.</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">short</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -294,6 +336,16 @@
           <t xml:space="preserve">Blister foil torn at one cavity on arrival. Capsule present and intact.</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Capsules 20 mg</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">short</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -339,6 +391,16 @@
           <t xml:space="preserve">Measuring cup missing from the carton.</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Oral Solution 100 ml</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -384,6 +446,16 @@
           <t xml:space="preserve">Carton crushed in transport. The shipping box was also damaged.</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -429,6 +501,16 @@
           <t xml:space="preserve">Customer reports a dark fibre in the cream after first opening of the tube. Sample requested.</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Cream 30 g</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -474,6 +556,16 @@
           <t xml:space="preserve">Two cartons in one shipment dented. Contents not affected.</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Capsules 20 mg</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -519,6 +611,16 @@
           <t xml:space="preserve">Patient leaflet missing from the carton.</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -562,6 +664,16 @@
       <c r="I12" t="inlineStr">
         <is>
           <t xml:space="preserve">Blister strip cracked across two cavities, one tablet broken. Customer asked for a call back on +49 30 5550 1234.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYN Tablets 50 mg</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>

</xml_diff>